<commit_message>
Add Beitar Ilit (BTR) and dedicated street processing script
- Added BTR to CITY_NAMES (Beitar Ilit)
- Created BTR_street_network_polygon.shp via dissolve + sliver fix
- batch_process_streets.py: dedicated street network processing script
  with full dissolve/repair/sliver-fix/hole-fill pipeline. Reusable
  for future cities. CLI supports processing all or specific cities.
- Regenerated urban forest analysis (40 cities) and street tree
  analysis (18 cities) including BTR
- BTR stats: 13,289 trees, median crown 4.9m (below national 6.1m)

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/street_trees_data.xlsx
+++ b/street_trees_data.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA18"/>
+  <dimension ref="A1:AA19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -640,7 +640,7 @@
         <v>21.73692744223754</v>
       </c>
       <c r="Z2" t="n">
-        <v>0.9323529411764706</v>
+        <v>0.9361111111111111</v>
       </c>
       <c r="AA2" t="n">
         <v>1</v>
@@ -729,7 +729,7 @@
         <v>23.15551659023469</v>
       </c>
       <c r="Z3" t="n">
-        <v>0.75</v>
+        <v>0.7638888888888888</v>
       </c>
       <c r="AA3" t="n">
         <v>2</v>
@@ -818,7 +818,7 @@
         <v>20.24832855778414</v>
       </c>
       <c r="Z4" t="n">
-        <v>0.7470588235294118</v>
+        <v>0.7611111111111112</v>
       </c>
       <c r="AA4" t="n">
         <v>3</v>
@@ -907,7 +907,7 @@
         <v>12.6040999359385</v>
       </c>
       <c r="Z5" t="n">
-        <v>0.7294117647058823</v>
+        <v>0.7444444444444444</v>
       </c>
       <c r="AA5" t="n">
         <v>4</v>
@@ -996,7 +996,7 @@
         <v>19.91738382099828</v>
       </c>
       <c r="Z6" t="n">
-        <v>0.711764705882353</v>
+        <v>0.7277777777777779</v>
       </c>
       <c r="AA6" t="n">
         <v>5</v>
@@ -1085,7 +1085,7 @@
         <v>11.32698412698413</v>
       </c>
       <c r="Z7" t="n">
-        <v>0.6588235294117648</v>
+        <v>0.6694444444444445</v>
       </c>
       <c r="AA7" t="n">
         <v>6</v>
@@ -1174,7 +1174,7 @@
         <v>11.22317990097194</v>
       </c>
       <c r="Z8" t="n">
-        <v>0.6323529411764706</v>
+        <v>0.6444444444444444</v>
       </c>
       <c r="AA8" t="n">
         <v>7</v>
@@ -1263,7 +1263,7 @@
         <v>26.50636293327709</v>
       </c>
       <c r="Z9" t="n">
-        <v>0.5647058823529412</v>
+        <v>0.5888888888888889</v>
       </c>
       <c r="AA9" t="n">
         <v>8</v>
@@ -1352,7 +1352,7 @@
         <v>16.70091441487722</v>
       </c>
       <c r="Z10" t="n">
-        <v>0.538235294117647</v>
+        <v>0.5638888888888889</v>
       </c>
       <c r="AA10" t="n">
         <v>9</v>
@@ -1441,7 +1441,7 @@
         <v>16.66106818945247</v>
       </c>
       <c r="Z11" t="n">
-        <v>0.511764705882353</v>
+        <v>0.5388888888888889</v>
       </c>
       <c r="AA11" t="n">
         <v>10</v>
@@ -1530,7 +1530,7 @@
         <v>20.66997518610422</v>
       </c>
       <c r="Z12" t="n">
-        <v>0.3705882352941176</v>
+        <v>0.4055555555555556</v>
       </c>
       <c r="AA12" t="n">
         <v>11</v>
@@ -1619,7 +1619,7 @@
         <v>32.15619166148102</v>
       </c>
       <c r="Z13" t="n">
-        <v>0.361764705882353</v>
+        <v>0.3972222222222222</v>
       </c>
       <c r="AA13" t="n">
         <v>12</v>
@@ -1708,7 +1708,7 @@
         <v>38.64099388806775</v>
       </c>
       <c r="Z14" t="n">
-        <v>0.3529411764705883</v>
+        <v>0.3666666666666667</v>
       </c>
       <c r="AA14" t="n">
         <v>13</v>
@@ -1797,7 +1797,7 @@
         <v>45.38963688290494</v>
       </c>
       <c r="Z15" t="n">
-        <v>0.3323529411764705</v>
+        <v>0.3472222222222223</v>
       </c>
       <c r="AA15" t="n">
         <v>14</v>
@@ -1886,7 +1886,7 @@
         <v>16.15384615384615</v>
       </c>
       <c r="Z16" t="n">
-        <v>0.3</v>
+        <v>0.3305555555555555</v>
       </c>
       <c r="AA16" t="n">
         <v>15</v>
@@ -1975,7 +1975,7 @@
         <v>22.21954161640531</v>
       </c>
       <c r="Z17" t="n">
-        <v>0.2558823529411765</v>
+        <v>0.2972222222222222</v>
       </c>
       <c r="AA17" t="n">
         <v>16</v>
@@ -2064,10 +2064,99 @@
         <v>39.0982087708462</v>
       </c>
       <c r="Z18" t="n">
-        <v>0.25</v>
+        <v>0.2694444444444444</v>
       </c>
       <c r="AA18" t="n">
         <v>17</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>BTR</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Beitar Ilit</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>2022_streets</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>2528</v>
+      </c>
+      <c r="E19" t="n">
+        <v>2268</v>
+      </c>
+      <c r="F19" t="n">
+        <v>1.114638447971781</v>
+      </c>
+      <c r="G19" t="n">
+        <v>5.096954113924051</v>
+      </c>
+      <c r="H19" t="n">
+        <v>5</v>
+      </c>
+      <c r="I19" t="n">
+        <v>1.721672463240113</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0.3377845718753448</v>
+      </c>
+      <c r="K19" t="n">
+        <v>2.399999999999999</v>
+      </c>
+      <c r="L19" t="n">
+        <v>3</v>
+      </c>
+      <c r="M19" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="N19" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="O19" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="P19" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="R19" t="n">
+        <v>0.8257511206595648</v>
+      </c>
+      <c r="S19" t="n">
+        <v>22.73386075949367</v>
+      </c>
+      <c r="T19" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="U19" t="n">
+        <v>80.22151898734177</v>
+      </c>
+      <c r="V19" t="n">
+        <v>4.846597633136096</v>
+      </c>
+      <c r="W19" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="X19" t="n">
+        <v>1.068037974683544</v>
+      </c>
+      <c r="Y19" t="n">
+        <v>30.0632911392405</v>
+      </c>
+      <c r="Z19" t="n">
+        <v>0.1472222222222222</v>
+      </c>
+      <c r="AA19" t="n">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -2081,7 +2170,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O18"/>
+  <dimension ref="A1:O19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2266,46 +2355,46 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BTY</t>
+          <t>BTR</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Bat Yam</t>
+          <t>Beitar Ilit</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>678</v>
+        <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>716</v>
+        <v>227</v>
       </c>
       <c r="E4" t="n">
-        <v>673</v>
+        <v>533</v>
       </c>
       <c r="F4" t="n">
-        <v>709</v>
+        <v>495</v>
       </c>
       <c r="G4" t="n">
-        <v>855</v>
+        <v>539</v>
       </c>
       <c r="H4" t="n">
-        <v>961</v>
+        <v>404</v>
       </c>
       <c r="I4" t="n">
-        <v>734</v>
+        <v>169</v>
       </c>
       <c r="J4" t="n">
-        <v>408</v>
+        <v>101</v>
       </c>
       <c r="K4" t="n">
-        <v>398</v>
+        <v>33</v>
       </c>
       <c r="L4" t="n">
-        <v>228</v>
+        <v>20</v>
       </c>
       <c r="M4" t="n">
-        <v>68</v>
+        <v>7</v>
       </c>
       <c r="N4" t="n">
         <v>0</v>
@@ -2317,46 +2406,46 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ELT</t>
+          <t>BTY</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Eilat</t>
+          <t>Bat Yam</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>678</v>
       </c>
       <c r="D5" t="n">
-        <v>296</v>
+        <v>716</v>
       </c>
       <c r="E5" t="n">
-        <v>625</v>
+        <v>673</v>
       </c>
       <c r="F5" t="n">
-        <v>682</v>
+        <v>709</v>
       </c>
       <c r="G5" t="n">
-        <v>858</v>
+        <v>855</v>
       </c>
       <c r="H5" t="n">
-        <v>691</v>
+        <v>961</v>
       </c>
       <c r="I5" t="n">
-        <v>387</v>
+        <v>734</v>
       </c>
       <c r="J5" t="n">
-        <v>298</v>
+        <v>408</v>
       </c>
       <c r="K5" t="n">
-        <v>148</v>
+        <v>398</v>
       </c>
       <c r="L5" t="n">
-        <v>135</v>
+        <v>228</v>
       </c>
       <c r="M5" t="n">
-        <v>25</v>
+        <v>68</v>
       </c>
       <c r="N5" t="n">
         <v>0</v>
@@ -2368,49 +2457,49 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>HAI</t>
+          <t>ELT</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Haifa</t>
+          <t>Eilat</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>2247</v>
+        <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>2418</v>
+        <v>296</v>
       </c>
       <c r="E6" t="n">
-        <v>2202</v>
+        <v>625</v>
       </c>
       <c r="F6" t="n">
-        <v>2469</v>
+        <v>682</v>
       </c>
       <c r="G6" t="n">
-        <v>3687</v>
+        <v>858</v>
       </c>
       <c r="H6" t="n">
-        <v>4859</v>
+        <v>691</v>
       </c>
       <c r="I6" t="n">
-        <v>4347</v>
+        <v>387</v>
       </c>
       <c r="J6" t="n">
-        <v>3294</v>
+        <v>298</v>
       </c>
       <c r="K6" t="n">
-        <v>1897</v>
+        <v>148</v>
       </c>
       <c r="L6" t="n">
-        <v>1511</v>
+        <v>135</v>
       </c>
       <c r="M6" t="n">
-        <v>700</v>
+        <v>25</v>
       </c>
       <c r="N6" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="O6" t="n">
         <v>0</v>
@@ -2419,253 +2508,253 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>HDS</t>
+          <t>HAI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Hod HaSharon</t>
+          <t>Haifa</t>
         </is>
       </c>
       <c r="C7" t="n">
+        <v>2247</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2418</v>
+      </c>
+      <c r="E7" t="n">
+        <v>2202</v>
+      </c>
+      <c r="F7" t="n">
+        <v>2469</v>
+      </c>
+      <c r="G7" t="n">
+        <v>3687</v>
+      </c>
+      <c r="H7" t="n">
+        <v>4859</v>
+      </c>
+      <c r="I7" t="n">
+        <v>4347</v>
+      </c>
+      <c r="J7" t="n">
+        <v>3294</v>
+      </c>
+      <c r="K7" t="n">
+        <v>1897</v>
+      </c>
+      <c r="L7" t="n">
+        <v>1511</v>
+      </c>
+      <c r="M7" t="n">
+        <v>700</v>
+      </c>
+      <c r="N7" t="n">
+        <v>25</v>
+      </c>
+      <c r="O7" t="n">
         <v>0</v>
-      </c>
-      <c r="D7" t="n">
-        <v>370</v>
-      </c>
-      <c r="E7" t="n">
-        <v>854</v>
-      </c>
-      <c r="F7" t="n">
-        <v>1099</v>
-      </c>
-      <c r="G7" t="n">
-        <v>1809</v>
-      </c>
-      <c r="H7" t="n">
-        <v>2511</v>
-      </c>
-      <c r="I7" t="n">
-        <v>1857</v>
-      </c>
-      <c r="J7" t="n">
-        <v>1152</v>
-      </c>
-      <c r="K7" t="n">
-        <v>625</v>
-      </c>
-      <c r="L7" t="n">
-        <v>440</v>
-      </c>
-      <c r="M7" t="n">
-        <v>180</v>
-      </c>
-      <c r="N7" t="n">
-        <v>8</v>
-      </c>
-      <c r="O7" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>HOL</t>
+          <t>HDS</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Holon</t>
+          <t>Hod HaSharon</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1258</v>
+        <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>1293</v>
+        <v>370</v>
       </c>
       <c r="E8" t="n">
-        <v>1219</v>
+        <v>854</v>
       </c>
       <c r="F8" t="n">
-        <v>1554</v>
+        <v>1099</v>
       </c>
       <c r="G8" t="n">
-        <v>1848</v>
+        <v>1809</v>
       </c>
       <c r="H8" t="n">
-        <v>2012</v>
+        <v>2511</v>
       </c>
       <c r="I8" t="n">
-        <v>1802</v>
+        <v>1857</v>
       </c>
       <c r="J8" t="n">
-        <v>1433</v>
+        <v>1152</v>
       </c>
       <c r="K8" t="n">
-        <v>912</v>
+        <v>625</v>
       </c>
       <c r="L8" t="n">
-        <v>681</v>
+        <v>440</v>
       </c>
       <c r="M8" t="n">
-        <v>210</v>
+        <v>180</v>
       </c>
       <c r="N8" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="O8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>HRZ</t>
+          <t>HOL</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Herzliya</t>
+          <t>Holon</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1290</v>
+        <v>1258</v>
       </c>
       <c r="D9" t="n">
-        <v>1287</v>
+        <v>1293</v>
       </c>
       <c r="E9" t="n">
-        <v>1239</v>
+        <v>1219</v>
       </c>
       <c r="F9" t="n">
-        <v>1543</v>
+        <v>1554</v>
       </c>
       <c r="G9" t="n">
-        <v>2556</v>
+        <v>1848</v>
       </c>
       <c r="H9" t="n">
-        <v>3295</v>
+        <v>2012</v>
       </c>
       <c r="I9" t="n">
-        <v>2850</v>
+        <v>1802</v>
       </c>
       <c r="J9" t="n">
-        <v>2303</v>
+        <v>1433</v>
       </c>
       <c r="K9" t="n">
-        <v>1130</v>
+        <v>912</v>
       </c>
       <c r="L9" t="n">
-        <v>1056</v>
+        <v>681</v>
       </c>
       <c r="M9" t="n">
-        <v>278</v>
+        <v>210</v>
       </c>
       <c r="N9" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="O9" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>KFS</t>
+          <t>HRZ</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Kfar Saba</t>
+          <t>Herzliya</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>942</v>
+        <v>1290</v>
       </c>
       <c r="D10" t="n">
-        <v>1030</v>
+        <v>1287</v>
       </c>
       <c r="E10" t="n">
-        <v>921</v>
+        <v>1239</v>
       </c>
       <c r="F10" t="n">
-        <v>1208</v>
+        <v>1543</v>
       </c>
       <c r="G10" t="n">
-        <v>1967</v>
+        <v>2556</v>
       </c>
       <c r="H10" t="n">
-        <v>2660</v>
+        <v>3295</v>
       </c>
       <c r="I10" t="n">
-        <v>2230</v>
+        <v>2850</v>
       </c>
       <c r="J10" t="n">
-        <v>1466</v>
+        <v>2303</v>
       </c>
       <c r="K10" t="n">
-        <v>1105</v>
+        <v>1130</v>
       </c>
       <c r="L10" t="n">
-        <v>690</v>
+        <v>1056</v>
       </c>
       <c r="M10" t="n">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="N10" t="n">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="O10" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>NSZ</t>
+          <t>KFS</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Ness Ziona</t>
+          <t>Kfar Saba</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0</v>
+        <v>942</v>
       </c>
       <c r="D11" t="n">
-        <v>392</v>
+        <v>1030</v>
       </c>
       <c r="E11" t="n">
-        <v>931</v>
+        <v>921</v>
       </c>
       <c r="F11" t="n">
-        <v>1148</v>
+        <v>1208</v>
       </c>
       <c r="G11" t="n">
-        <v>1694</v>
+        <v>1967</v>
       </c>
       <c r="H11" t="n">
-        <v>1886</v>
+        <v>2660</v>
       </c>
       <c r="I11" t="n">
-        <v>1008</v>
+        <v>2230</v>
       </c>
       <c r="J11" t="n">
-        <v>573</v>
+        <v>1466</v>
       </c>
       <c r="K11" t="n">
-        <v>279</v>
+        <v>1105</v>
       </c>
       <c r="L11" t="n">
-        <v>213</v>
+        <v>690</v>
       </c>
       <c r="M11" t="n">
-        <v>66</v>
+        <v>274</v>
       </c>
       <c r="N11" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="O11" t="n">
         <v>0</v>
@@ -2674,151 +2763,151 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>NTN</t>
+          <t>NSZ</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Netanya</t>
+          <t>Ness Ziona</t>
         </is>
       </c>
       <c r="C12" t="n">
         <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>986</v>
+        <v>392</v>
       </c>
       <c r="E12" t="n">
-        <v>2265</v>
+        <v>931</v>
       </c>
       <c r="F12" t="n">
-        <v>2615</v>
+        <v>1148</v>
       </c>
       <c r="G12" t="n">
-        <v>3700</v>
+        <v>1694</v>
       </c>
       <c r="H12" t="n">
-        <v>3685</v>
+        <v>1886</v>
       </c>
       <c r="I12" t="n">
-        <v>2699</v>
+        <v>1008</v>
       </c>
       <c r="J12" t="n">
-        <v>1570</v>
+        <v>573</v>
       </c>
       <c r="K12" t="n">
-        <v>947</v>
+        <v>279</v>
       </c>
       <c r="L12" t="n">
-        <v>728</v>
+        <v>213</v>
       </c>
       <c r="M12" t="n">
-        <v>225</v>
+        <v>66</v>
       </c>
       <c r="N12" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="O12" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>NTV</t>
+          <t>NTN</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Netivot</t>
+          <t>Netanya</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>407</v>
+        <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>436</v>
+        <v>986</v>
       </c>
       <c r="E13" t="n">
-        <v>423</v>
+        <v>2265</v>
       </c>
       <c r="F13" t="n">
-        <v>480</v>
+        <v>2615</v>
       </c>
       <c r="G13" t="n">
-        <v>471</v>
+        <v>3700</v>
       </c>
       <c r="H13" t="n">
-        <v>406</v>
+        <v>3685</v>
       </c>
       <c r="I13" t="n">
-        <v>257</v>
+        <v>2699</v>
       </c>
       <c r="J13" t="n">
-        <v>131</v>
+        <v>1570</v>
       </c>
       <c r="K13" t="n">
-        <v>107</v>
+        <v>947</v>
       </c>
       <c r="L13" t="n">
-        <v>71</v>
+        <v>728</v>
       </c>
       <c r="M13" t="n">
-        <v>47</v>
+        <v>225</v>
       </c>
       <c r="N13" t="n">
-        <v>2</v>
+        <v>42</v>
       </c>
       <c r="O13" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>PHK</t>
+          <t>NTV</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Pardes Hanna-Karkur</t>
+          <t>Netivot</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0</v>
+        <v>407</v>
       </c>
       <c r="D14" t="n">
-        <v>272</v>
+        <v>436</v>
       </c>
       <c r="E14" t="n">
-        <v>620</v>
+        <v>423</v>
       </c>
       <c r="F14" t="n">
-        <v>868</v>
+        <v>480</v>
       </c>
       <c r="G14" t="n">
-        <v>1176</v>
+        <v>471</v>
       </c>
       <c r="H14" t="n">
-        <v>1722</v>
+        <v>406</v>
       </c>
       <c r="I14" t="n">
-        <v>1306</v>
+        <v>257</v>
       </c>
       <c r="J14" t="n">
-        <v>965</v>
+        <v>131</v>
       </c>
       <c r="K14" t="n">
-        <v>449</v>
+        <v>107</v>
       </c>
       <c r="L14" t="n">
-        <v>399</v>
+        <v>71</v>
       </c>
       <c r="M14" t="n">
-        <v>95</v>
+        <v>47</v>
       </c>
       <c r="N14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O14" t="n">
         <v>0</v>
@@ -2827,49 +2916,49 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PTV</t>
+          <t>PHK</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Petah Tikva</t>
+          <t>Pardes Hanna-Karkur</t>
         </is>
       </c>
       <c r="C15" t="n">
         <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>724</v>
+        <v>272</v>
       </c>
       <c r="E15" t="n">
-        <v>1637</v>
+        <v>620</v>
       </c>
       <c r="F15" t="n">
-        <v>2066</v>
+        <v>868</v>
       </c>
       <c r="G15" t="n">
-        <v>3285</v>
+        <v>1176</v>
       </c>
       <c r="H15" t="n">
-        <v>3640</v>
+        <v>1722</v>
       </c>
       <c r="I15" t="n">
-        <v>2695</v>
+        <v>1306</v>
       </c>
       <c r="J15" t="n">
-        <v>1833</v>
+        <v>965</v>
       </c>
       <c r="K15" t="n">
-        <v>1422</v>
+        <v>449</v>
       </c>
       <c r="L15" t="n">
-        <v>1111</v>
+        <v>399</v>
       </c>
       <c r="M15" t="n">
-        <v>310</v>
+        <v>95</v>
       </c>
       <c r="N15" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="O15" t="n">
         <v>0</v>
@@ -2878,49 +2967,49 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>RAN</t>
+          <t>PTV</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Raanana</t>
+          <t>Petah Tikva</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>742</v>
+        <v>0</v>
       </c>
       <c r="D16" t="n">
-        <v>852</v>
+        <v>724</v>
       </c>
       <c r="E16" t="n">
-        <v>886</v>
+        <v>1637</v>
       </c>
       <c r="F16" t="n">
-        <v>1371</v>
+        <v>2066</v>
       </c>
       <c r="G16" t="n">
-        <v>2549</v>
+        <v>3285</v>
       </c>
       <c r="H16" t="n">
-        <v>2897</v>
+        <v>3640</v>
       </c>
       <c r="I16" t="n">
-        <v>2431</v>
+        <v>2695</v>
       </c>
       <c r="J16" t="n">
-        <v>1569</v>
+        <v>1833</v>
       </c>
       <c r="K16" t="n">
-        <v>895</v>
+        <v>1422</v>
       </c>
       <c r="L16" t="n">
-        <v>543</v>
+        <v>1111</v>
       </c>
       <c r="M16" t="n">
-        <v>143</v>
+        <v>310</v>
       </c>
       <c r="N16" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="O16" t="n">
         <v>0</v>
@@ -2929,49 +3018,49 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SDR</t>
+          <t>RAN</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Sderot</t>
+          <t>Raanana</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>715</v>
+        <v>742</v>
       </c>
       <c r="D17" t="n">
-        <v>828</v>
+        <v>852</v>
       </c>
       <c r="E17" t="n">
-        <v>682</v>
+        <v>886</v>
       </c>
       <c r="F17" t="n">
-        <v>702</v>
+        <v>1371</v>
       </c>
       <c r="G17" t="n">
-        <v>593</v>
+        <v>2549</v>
       </c>
       <c r="H17" t="n">
-        <v>484</v>
+        <v>2897</v>
       </c>
       <c r="I17" t="n">
-        <v>316</v>
+        <v>2431</v>
       </c>
       <c r="J17" t="n">
-        <v>209</v>
+        <v>1569</v>
       </c>
       <c r="K17" t="n">
-        <v>142</v>
+        <v>895</v>
       </c>
       <c r="L17" t="n">
-        <v>150</v>
+        <v>543</v>
       </c>
       <c r="M17" t="n">
-        <v>60</v>
+        <v>143</v>
       </c>
       <c r="N17" t="n">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="O17" t="n">
         <v>0</v>
@@ -2980,51 +3069,102 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>SDR</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Sderot</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>715</v>
+      </c>
+      <c r="D18" t="n">
+        <v>828</v>
+      </c>
+      <c r="E18" t="n">
+        <v>682</v>
+      </c>
+      <c r="F18" t="n">
+        <v>702</v>
+      </c>
+      <c r="G18" t="n">
+        <v>593</v>
+      </c>
+      <c r="H18" t="n">
+        <v>484</v>
+      </c>
+      <c r="I18" t="n">
+        <v>316</v>
+      </c>
+      <c r="J18" t="n">
+        <v>209</v>
+      </c>
+      <c r="K18" t="n">
+        <v>142</v>
+      </c>
+      <c r="L18" t="n">
+        <v>150</v>
+      </c>
+      <c r="M18" t="n">
+        <v>60</v>
+      </c>
+      <c r="N18" t="n">
+        <v>20</v>
+      </c>
+      <c r="O18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>TLV</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>Tel Aviv</t>
         </is>
       </c>
-      <c r="C18" t="n">
+      <c r="C19" t="n">
         <v>4145</v>
       </c>
-      <c r="D18" t="n">
+      <c r="D19" t="n">
         <v>4512</v>
       </c>
-      <c r="E18" t="n">
+      <c r="E19" t="n">
         <v>4213</v>
       </c>
-      <c r="F18" t="n">
+      <c r="F19" t="n">
         <v>4904</v>
       </c>
-      <c r="G18" t="n">
+      <c r="G19" t="n">
         <v>7368</v>
       </c>
-      <c r="H18" t="n">
+      <c r="H19" t="n">
         <v>8749</v>
       </c>
-      <c r="I18" t="n">
+      <c r="I19" t="n">
         <v>8108</v>
       </c>
-      <c r="J18" t="n">
+      <c r="J19" t="n">
         <v>6884</v>
       </c>
-      <c r="K18" t="n">
+      <c r="K19" t="n">
         <v>4463</v>
       </c>
-      <c r="L18" t="n">
+      <c r="L19" t="n">
         <v>4316</v>
       </c>
-      <c r="M18" t="n">
+      <c r="M19" t="n">
         <v>1327</v>
       </c>
-      <c r="N18" t="n">
+      <c r="N19" t="n">
         <v>156</v>
       </c>
-      <c r="O18" t="n">
+      <c r="O19" t="n">
         <v>63</v>
       </c>
     </row>
@@ -3039,7 +3179,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3147,28 +3287,28 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BTY</t>
+          <t>BTR</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Bat Yam</t>
+          <t>Beitar Ilit</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>32.15619166148102</v>
+        <v>30.0632911392405</v>
       </c>
       <c r="D4" t="n">
-        <v>24.33105164903547</v>
+        <v>40.90189873417722</v>
       </c>
       <c r="E4" t="n">
-        <v>26.36901057871811</v>
+        <v>22.66613924050633</v>
       </c>
       <c r="F4" t="n">
-        <v>12.53889234598631</v>
+        <v>5.300632911392404</v>
       </c>
       <c r="G4" t="n">
-        <v>4.604853764779091</v>
+        <v>1.068037974683544</v>
       </c>
       <c r="H4" t="n">
         <v>0</v>
@@ -3177,28 +3317,28 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ELT</t>
+          <t>BTY</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Eilat</t>
+          <t>Bat Yam</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>22.21954161640531</v>
+        <v>32.15619166148102</v>
       </c>
       <c r="D5" t="n">
-        <v>37.15319662243667</v>
+        <v>24.33105164903547</v>
       </c>
       <c r="E5" t="n">
-        <v>26.00723763570567</v>
+        <v>26.36901057871811</v>
       </c>
       <c r="F5" t="n">
-        <v>10.7599517490953</v>
+        <v>12.53889234598631</v>
       </c>
       <c r="G5" t="n">
-        <v>3.860072376357056</v>
+        <v>4.604853764779091</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
@@ -3207,390 +3347,420 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>HAI</t>
+          <t>ELT</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Haifa</t>
+          <t>Eilat</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>23.15551659023469</v>
+        <v>22.21954161640531</v>
       </c>
       <c r="D6" t="n">
-        <v>20.75802535743189</v>
+        <v>37.15319662243667</v>
       </c>
       <c r="E6" t="n">
-        <v>31.04262206636094</v>
+        <v>26.00723763570567</v>
       </c>
       <c r="F6" t="n">
-        <v>17.50404639870515</v>
+        <v>10.7599517490953</v>
       </c>
       <c r="G6" t="n">
-        <v>7.455489614243324</v>
+        <v>3.860072376357056</v>
       </c>
       <c r="H6" t="n">
-        <v>0.08429997302400864</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>HDS</t>
+          <t>HAI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Hod HaSharon</t>
+          <t>Haifa</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>11.22317990097194</v>
+        <v>23.15551659023469</v>
       </c>
       <c r="D7" t="n">
-        <v>26.66422152943334</v>
+        <v>20.75802535743189</v>
       </c>
       <c r="E7" t="n">
-        <v>40.05134788189987</v>
+        <v>31.04262206636094</v>
       </c>
       <c r="F7" t="n">
-        <v>16.29378323858427</v>
+        <v>17.50404639870515</v>
       </c>
       <c r="G7" t="n">
-        <v>5.684944067485788</v>
+        <v>7.455489614243324</v>
       </c>
       <c r="H7" t="n">
-        <v>0.0825233816247937</v>
+        <v>0.08429997302400864</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>HOL</t>
+          <t>HDS</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Holon</t>
+          <t>Hod HaSharon</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>26.50636293327709</v>
+        <v>11.22317990097194</v>
       </c>
       <c r="D8" t="n">
-        <v>23.91900442944527</v>
+        <v>26.66422152943334</v>
       </c>
       <c r="E8" t="n">
-        <v>26.81572101525698</v>
+        <v>40.05134788189987</v>
       </c>
       <c r="F8" t="n">
-        <v>16.48737959642832</v>
+        <v>16.29378323858427</v>
       </c>
       <c r="G8" t="n">
-        <v>6.264501160092808</v>
+        <v>5.684944067485788</v>
       </c>
       <c r="H8" t="n">
-        <v>0.007030865499542995</v>
+        <v>0.0825233816247937</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>HRZ</t>
+          <t>HOL</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Herzliya</t>
+          <t>Holon</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>20.24832855778414</v>
+        <v>26.50636293327709</v>
       </c>
       <c r="D9" t="n">
-        <v>21.74997346917118</v>
+        <v>23.91900442944527</v>
       </c>
       <c r="E9" t="n">
-        <v>32.6063886235806</v>
+        <v>26.81572101525698</v>
       </c>
       <c r="F9" t="n">
-        <v>18.21606706993527</v>
+        <v>16.48737959642832</v>
       </c>
       <c r="G9" t="n">
-        <v>7.078425130001061</v>
+        <v>6.264501160092808</v>
       </c>
       <c r="H9" t="n">
-        <v>0.1008171495277513</v>
+        <v>0.007030865499542995</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>KFS</t>
+          <t>HRZ</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Kfar Saba</t>
+          <t>Herzliya</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>19.91738382099828</v>
+        <v>20.24832855778414</v>
       </c>
       <c r="D10" t="n">
-        <v>21.85886402753873</v>
+        <v>21.74997346917118</v>
       </c>
       <c r="E10" t="n">
-        <v>33.66609294320138</v>
+        <v>32.6063886235806</v>
       </c>
       <c r="F10" t="n">
-        <v>17.70051635111876</v>
+        <v>18.21606706993527</v>
       </c>
       <c r="G10" t="n">
-        <v>6.6368330464716</v>
+        <v>7.078425130001061</v>
       </c>
       <c r="H10" t="n">
-        <v>0.2203098106712565</v>
+        <v>0.1008171495277513</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>NSZ</t>
+          <t>KFS</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Ness Ziona</t>
+          <t>Kfar Saba</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>16.15384615384615</v>
+        <v>19.91738382099828</v>
       </c>
       <c r="D11" t="n">
-        <v>34.7008547008547</v>
+        <v>21.85886402753873</v>
       </c>
       <c r="E11" t="n">
-        <v>35.33577533577534</v>
+        <v>33.66609294320138</v>
       </c>
       <c r="F11" t="n">
-        <v>10.4029304029304</v>
+        <v>17.70051635111876</v>
       </c>
       <c r="G11" t="n">
-        <v>3.406593406593406</v>
+        <v>6.6368330464716</v>
       </c>
       <c r="H11" t="n">
-        <v>0</v>
+        <v>0.2203098106712565</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>NTN</t>
+          <t>NSZ</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Netanya</t>
+          <t>Ness Ziona</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>16.70091441487722</v>
+        <v>16.15384615384615</v>
       </c>
       <c r="D12" t="n">
-        <v>32.44117949244838</v>
+        <v>34.7008547008547</v>
       </c>
       <c r="E12" t="n">
-        <v>32.79564368642762</v>
+        <v>35.33577533577534</v>
       </c>
       <c r="F12" t="n">
-        <v>12.9302373368951</v>
+        <v>10.4029304029304</v>
       </c>
       <c r="G12" t="n">
-        <v>4.89571560669886</v>
+        <v>3.406593406593406</v>
       </c>
       <c r="H12" t="n">
-        <v>0.2363094626528306</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>NTV</t>
+          <t>NTN</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Netivot</t>
+          <t>Netanya</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>39.0982087708462</v>
+        <v>16.70091441487722</v>
       </c>
       <c r="D13" t="n">
-        <v>29.36998147004324</v>
+        <v>32.44117949244838</v>
       </c>
       <c r="E13" t="n">
-        <v>20.47560222359481</v>
+        <v>32.79564368642762</v>
       </c>
       <c r="F13" t="n">
-        <v>7.350216182828907</v>
+        <v>12.9302373368951</v>
       </c>
       <c r="G13" t="n">
-        <v>3.644224830142063</v>
+        <v>4.89571560669886</v>
       </c>
       <c r="H13" t="n">
-        <v>0.06176652254478073</v>
+        <v>0.2363094626528306</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>PHK</t>
+          <t>NTV</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Pardes Hanna-Karkur</t>
+          <t>Netivot</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>11.32698412698413</v>
+        <v>39.0982087708462</v>
       </c>
       <c r="D14" t="n">
-        <v>25.95555555555556</v>
+        <v>29.36998147004324</v>
       </c>
       <c r="E14" t="n">
-        <v>38.45079365079365</v>
+        <v>20.47560222359481</v>
       </c>
       <c r="F14" t="n">
-        <v>17.95555555555556</v>
+        <v>7.350216182828907</v>
       </c>
       <c r="G14" t="n">
-        <v>6.273015873015873</v>
+        <v>3.644224830142063</v>
       </c>
       <c r="H14" t="n">
-        <v>0.0380952380952381</v>
+        <v>0.06176652254478073</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PTV</t>
+          <t>PHK</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Petah Tikva</t>
+          <t>Pardes Hanna-Karkur</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>12.6040999359385</v>
+        <v>11.32698412698413</v>
       </c>
       <c r="D15" t="n">
-        <v>28.56609011317531</v>
+        <v>25.95555555555556</v>
       </c>
       <c r="E15" t="n">
-        <v>33.81913303437967</v>
+        <v>38.45079365079365</v>
       </c>
       <c r="F15" t="n">
-        <v>17.37668161434978</v>
+        <v>17.95555555555556</v>
       </c>
       <c r="G15" t="n">
-        <v>7.58594917787743</v>
+        <v>6.273015873015873</v>
       </c>
       <c r="H15" t="n">
-        <v>0.04804612427930814</v>
+        <v>0.0380952380952381</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>RAN</t>
+          <t>PTV</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Raanana</t>
+          <t>Petah Tikva</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>16.66106818945247</v>
+        <v>12.6040999359385</v>
       </c>
       <c r="D16" t="n">
-        <v>26.33523681558616</v>
+        <v>28.56609011317531</v>
       </c>
       <c r="E16" t="n">
-        <v>35.79442391669465</v>
+        <v>33.81913303437967</v>
       </c>
       <c r="F16" t="n">
-        <v>16.55357742693987</v>
+        <v>17.37668161434978</v>
       </c>
       <c r="G16" t="n">
-        <v>4.608666442727579</v>
+        <v>7.58594917787743</v>
       </c>
       <c r="H16" t="n">
-        <v>0.047027208599261</v>
+        <v>0.04804612427930814</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SDR</t>
+          <t>RAN</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Sderot</t>
+          <t>Raanana</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>45.38963688290494</v>
+        <v>16.66106818945247</v>
       </c>
       <c r="D17" t="n">
-        <v>26.41778865769074</v>
+        <v>26.33523681558616</v>
       </c>
       <c r="E17" t="n">
-        <v>16.31986944104447</v>
+        <v>35.79442391669465</v>
       </c>
       <c r="F17" t="n">
-        <v>7.160342717258263</v>
+        <v>16.55357742693987</v>
       </c>
       <c r="G17" t="n">
-        <v>4.283965728274174</v>
+        <v>4.608666442727579</v>
       </c>
       <c r="H17" t="n">
-        <v>0.4283965728274173</v>
+        <v>0.047027208599261</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>SDR</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Sderot</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>45.38963688290494</v>
+      </c>
+      <c r="D18" t="n">
+        <v>26.41778865769074</v>
+      </c>
+      <c r="E18" t="n">
+        <v>16.31986944104447</v>
+      </c>
+      <c r="F18" t="n">
+        <v>7.160342717258263</v>
+      </c>
+      <c r="G18" t="n">
+        <v>4.283965728274174</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0.4283965728274173</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>TLV</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>Tel Aviv</t>
         </is>
       </c>
-      <c r="C18" t="n">
+      <c r="C19" t="n">
         <v>21.73692744223754</v>
       </c>
-      <c r="D18" t="n">
+      <c r="D19" t="n">
         <v>20.72692879340629</v>
       </c>
-      <c r="E18" t="n">
+      <c r="E19" t="n">
         <v>28.47081475476287</v>
       </c>
-      <c r="F18" t="n">
+      <c r="F19" t="n">
         <v>19.1646399135252</v>
       </c>
-      <c r="G18" t="n">
+      <c r="G19" t="n">
         <v>9.530806647750303</v>
       </c>
-      <c r="H18" t="n">
+      <c r="H19" t="n">
         <v>0.3698824483177949</v>
       </c>
     </row>
@@ -3627,7 +3797,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>264288</v>
+        <v>266816</v>
       </c>
     </row>
     <row r="3">
@@ -3637,7 +3807,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>175410</v>
+        <v>177678</v>
       </c>
     </row>
     <row r="4">
@@ -3647,7 +3817,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5">
@@ -3657,7 +3827,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>6.08</v>
+        <v>6.07</v>
       </c>
     </row>
     <row r="6">
@@ -3667,7 +3837,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>6.17</v>
+        <v>6.15</v>
       </c>
     </row>
     <row r="7">
@@ -3677,7 +3847,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>6.7</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="8">
@@ -3687,7 +3857,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>22.2</v>
+        <v>22.3</v>
       </c>
     </row>
   </sheetData>
@@ -3731,7 +3901,7 @@
         <v>15655</v>
       </c>
       <c r="C2" t="n">
-        <v>5.923507109722044</v>
+        <v>5.867383270742915</v>
       </c>
     </row>
     <row r="3">
@@ -3741,10 +3911,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>20097</v>
+        <v>20324</v>
       </c>
       <c r="C3" t="n">
-        <v>7.604262049446434</v>
+        <v>7.617291446475822</v>
       </c>
     </row>
     <row r="4">
@@ -3754,10 +3924,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>22980</v>
+        <v>23513</v>
       </c>
       <c r="C4" t="n">
-        <v>8.695125734999205</v>
+        <v>8.812506090385062</v>
       </c>
     </row>
     <row r="5">
@@ -3767,10 +3937,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>27232</v>
+        <v>27727</v>
       </c>
       <c r="C5" t="n">
-        <v>10.30398886055258</v>
+        <v>10.39188348437488</v>
       </c>
     </row>
     <row r="6">
@@ -3780,10 +3950,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>38808</v>
+        <v>39347</v>
       </c>
       <c r="C6" t="n">
-        <v>14.6840922334138</v>
+        <v>14.74697729504449</v>
       </c>
     </row>
     <row r="7">
@@ -3793,10 +3963,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>44377</v>
+        <v>44781</v>
       </c>
       <c r="C7" t="n">
-        <v>16.79127914456309</v>
+        <v>16.78360205986193</v>
       </c>
     </row>
     <row r="8">
@@ -3806,10 +3976,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>35730</v>
+        <v>35899</v>
       </c>
       <c r="C8" t="n">
-        <v>13.51944484384341</v>
+        <v>13.45469128306611</v>
       </c>
     </row>
     <row r="9">
@@ -3819,10 +3989,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>25791</v>
+        <v>25892</v>
       </c>
       <c r="C9" t="n">
-        <v>9.758746206760858</v>
+        <v>9.704138463498916</v>
       </c>
     </row>
     <row r="10">
@@ -3832,10 +4002,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>15939</v>
+        <v>15972</v>
       </c>
       <c r="C10" t="n">
-        <v>6.03096645300924</v>
+        <v>5.986192628572714</v>
       </c>
     </row>
     <row r="11">
@@ -3845,10 +4015,10 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>13038</v>
+        <v>13058</v>
       </c>
       <c r="C11" t="n">
-        <v>4.933291964008688</v>
+        <v>4.894046039563142</v>
       </c>
     </row>
     <row r="12">
@@ -3858,10 +4028,10 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>4244</v>
+        <v>4251</v>
       </c>
       <c r="C12" t="n">
-        <v>1.605836101798809</v>
+        <v>1.593244732285412</v>
       </c>
     </row>
     <row r="13">
@@ -3874,7 +4044,7 @@
         <v>320</v>
       </c>
       <c r="C13" t="n">
-        <v>0.1210809501827566</v>
+        <v>0.1199337366105227</v>
       </c>
     </row>
     <row r="14">
@@ -3887,7 +4057,7 @@
         <v>75</v>
       </c>
       <c r="C14" t="n">
-        <v>0.02837834769908357</v>
+        <v>0.02810946951809125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>